<commit_message>
chore: update configuration, test scripts, and data files
</commit_message>
<xml_diff>
--- a/Informasi Kontak (Jawaban).xlsx
+++ b/Informasi Kontak (Jawaban).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Ruang-Tenang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F976D24B-0AFC-4372-8046-383EFBB49BD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF43C0FD-7F28-4D2B-A560-8098A6424722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="182">
   <si>
     <t>Timestamp</t>
   </si>
@@ -548,6 +548,27 @@
   </si>
   <si>
     <t>Bukti Follow Akun Instagram "Ruang Tenang Kendari" https://www.instagram.com/ruangtenang.community?igsh=MTNyOW90N2x0bzdjeA==</t>
+  </si>
+  <si>
+    <t>Eky</t>
+  </si>
+  <si>
+    <t>Gold 200K</t>
+  </si>
+  <si>
+    <t>Silver</t>
+  </si>
+  <si>
+    <t>6285254438227</t>
+  </si>
+  <si>
+    <t>+6285254438227</t>
+  </si>
+  <si>
+    <t>Ely Ermawati tes salah</t>
+  </si>
+  <si>
+    <t>Eky Sulis</t>
   </si>
 </sst>
 </file>
@@ -583,12 +604,24 @@
       <name val="Roboto"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF8F9FA"/>
+        <bgColor rgb="FFF8F9FA"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -603,7 +636,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -625,6 +658,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -986,12 +1025,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="18.90625" customWidth="1"/>
-    <col min="3" max="3" width="29.81640625" customWidth="1"/>
-    <col min="4" max="4" width="30.08984375" customWidth="1"/>
+    <col min="1" max="1" width="18.90625" customWidth="1"/>
+    <col min="2" max="3" width="29.81640625" customWidth="1"/>
+    <col min="4" max="4" width="33.90625" customWidth="1"/>
     <col min="5" max="9" width="18.90625" customWidth="1"/>
     <col min="10" max="10" width="20.7265625" customWidth="1"/>
     <col min="11" max="11" width="29.36328125" customWidth="1"/>
@@ -2493,6 +2532,314 @@
         <v>15</v>
       </c>
       <c r="N34" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" s="3">
+        <v>350</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I35" s="3">
+        <v>3</v>
+      </c>
+      <c r="J35" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N35" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E36" s="3">
+        <v>3</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H36" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I36" s="3">
+        <v>3</v>
+      </c>
+      <c r="J36" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K36" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M36" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N36" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" s="3">
+        <v>3</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I37" s="3">
+        <v>3</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K37" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N37" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B38" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>178</v>
+      </c>
+      <c r="E38" s="3">
+        <v>3</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I38" s="3">
+        <v>3</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K38" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L38" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M38" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="E39" s="3">
+        <v>3</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H39" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I39" s="3">
+        <v>3</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K39" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L39" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N39" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>46208.502451967594</v>
+      </c>
+      <c r="B40" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="E40" s="3">
+        <v>35</v>
+      </c>
+      <c r="F40" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G40" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="I40" s="3">
+        <v>1</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K40" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="L40" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="M40" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N40" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>46146.267447141203</v>
+      </c>
+      <c r="B41" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="8">
+        <v>85253822700</v>
+      </c>
+      <c r="E41" s="3">
+        <v>3</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G41" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="H41" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="I41" s="3">
+        <v>3</v>
+      </c>
+      <c r="J41" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K41" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="L41" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="M41" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N41" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2533,10 +2880,24 @@
     <hyperlink ref="K34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
     <hyperlink ref="M2" r:id="rId34" xr:uid="{0BE99F97-4218-4402-9D78-2E10BC4B924E}"/>
     <hyperlink ref="M3:M34" r:id="rId35" display="https://drive.google.com/open?id=1ncLerrEwpsR8w5xf8SSXG334E7fOu2R-" xr:uid="{3D388301-D9F2-42DA-A9C0-AABA62A48F07}"/>
+    <hyperlink ref="K35" r:id="rId36" xr:uid="{ACC58351-468A-4939-8ADD-0A99AD034A4C}"/>
+    <hyperlink ref="M35" r:id="rId37" xr:uid="{51268971-6898-4368-8216-B980E5B32BA4}"/>
+    <hyperlink ref="K36" r:id="rId38" xr:uid="{FB207ECB-910A-46DC-B96E-86A5CA0E2842}"/>
+    <hyperlink ref="M36" r:id="rId39" xr:uid="{4F23D56C-A79E-4957-B716-1C96D53704FE}"/>
+    <hyperlink ref="K37" r:id="rId40" xr:uid="{BE5B597F-7643-44C1-909D-533625A1E4AB}"/>
+    <hyperlink ref="M37" r:id="rId41" xr:uid="{9CE496CB-4FB2-49D1-B29F-60A57BF26F9E}"/>
+    <hyperlink ref="K38" r:id="rId42" xr:uid="{B679085D-5408-4DBF-9552-22C63BDCE08C}"/>
+    <hyperlink ref="M38" r:id="rId43" xr:uid="{F5B1B155-0DD2-49EE-BC05-C72A1B03D595}"/>
+    <hyperlink ref="K39" r:id="rId44" xr:uid="{E4C20335-B77C-44A9-AFFF-DBA969766DCF}"/>
+    <hyperlink ref="M39" r:id="rId45" xr:uid="{7F27F93F-40BF-43A3-94C3-0397E3BCBA49}"/>
+    <hyperlink ref="K40" r:id="rId46" xr:uid="{894FE79F-F7F3-401E-97D8-A3F032BD13D1}"/>
+    <hyperlink ref="M40" r:id="rId47" xr:uid="{A8DE7F3A-0698-4A9F-B94C-8857CE31C467}"/>
+    <hyperlink ref="K41" r:id="rId48" xr:uid="{A902B6BA-8088-4ED0-9FA5-B0B94025846C}"/>
+    <hyperlink ref="M41" r:id="rId49" xr:uid="{018ECE75-35A0-4D9B-8718-276209FBE571}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId36"/>
+    <tablePart r:id="rId50"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix bug import logic
</commit_message>
<xml_diff>
--- a/Informasi Kontak (Jawaban).xlsx
+++ b/Informasi Kontak (Jawaban).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Ruang-Tenang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF43C0FD-7F28-4D2B-A560-8098A6424722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC1366E-38E0-407E-BE5A-BE04AEA3B50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="168">
   <si>
     <t>Timestamp</t>
   </si>
@@ -500,33 +500,6 @@
     <t>Instagram</t>
   </si>
   <si>
-    <t>Ely Ermawati</t>
-  </si>
-  <si>
-    <t>elhycancer23@gmail.com</t>
-  </si>
-  <si>
-    <t>082322233342</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1fw6y2LH44NLyyqoT26yoQCtw1D1bqqKL</t>
-  </si>
-  <si>
-    <t>Hasmiranti</t>
-  </si>
-  <si>
-    <t>miranfaqih@gmail.com</t>
-  </si>
-  <si>
-    <t>085282011949</t>
-  </si>
-  <si>
-    <t>https://drive.google.com/open?id=1f8pjkBgnfjilxDne0o4e6zotLm9eteQS</t>
-  </si>
-  <si>
-    <t>Kesembuhan mental</t>
-  </si>
-  <si>
     <t>No. WhatsApp (Awalan nomor harus  +62)
 *</t>
   </si>
@@ -550,25 +523,10 @@
     <t>Bukti Follow Akun Instagram "Ruang Tenang Kendari" https://www.instagram.com/ruangtenang.community?igsh=MTNyOW90N2x0bzdjeA==</t>
   </si>
   <si>
-    <t>Eky</t>
-  </si>
-  <si>
-    <t>Gold 200K</t>
-  </si>
-  <si>
-    <t>Silver</t>
-  </si>
-  <si>
-    <t>6285254438227</t>
-  </si>
-  <si>
-    <t>+6285254438227</t>
-  </si>
-  <si>
-    <t>Ely Ermawati tes salah</t>
-  </si>
-  <si>
-    <t>Eky Sulis</t>
+    <t>IkhsandduinRezki</t>
+  </si>
+  <si>
+    <t>Ikhsanuddin@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -578,7 +536,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -603,25 +561,20 @@
       <color rgb="FF0000FF"/>
       <name val="Roboto"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF8F9FA"/>
-        <bgColor rgb="FFF8F9FA"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -633,10 +586,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -659,14 +613,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="8">
@@ -803,7 +755,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:N34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:N32">
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Nama Lengkap"/>
@@ -1025,7 +977,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
@@ -1050,7 +1002,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
@@ -1062,7 +1014,7 @@
         <v>5</v>
       </c>
       <c r="H1" s="7" t="s">
-        <v>169</v>
+        <v>160</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>6</v>
@@ -1071,13 +1023,13 @@
         <v>7</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>9</v>
@@ -1103,10 +1055,10 @@
         <v>12</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I2" s="3">
         <v>3</v>
@@ -1147,10 +1099,10 @@
         <v>12</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I3" s="3">
         <v>1</v>
@@ -1191,10 +1143,10 @@
         <v>12</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I4" s="3">
         <v>2</v>
@@ -1235,10 +1187,10 @@
         <v>12</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I5" s="3">
         <v>1</v>
@@ -1279,10 +1231,10 @@
         <v>12</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I6" s="3">
         <v>1</v>
@@ -1323,10 +1275,10 @@
         <v>12</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I7" s="3">
         <v>3</v>
@@ -1367,10 +1319,10 @@
         <v>12</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I8" s="3">
         <v>1</v>
@@ -1411,10 +1363,10 @@
         <v>12</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I9" s="3">
         <v>1</v>
@@ -1455,10 +1407,10 @@
         <v>12</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I10" s="3">
         <v>1</v>
@@ -1499,10 +1451,10 @@
         <v>12</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I11" s="3">
         <v>2</v>
@@ -1543,10 +1495,10 @@
         <v>12</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
       <c r="I12" s="3">
         <v>1</v>
@@ -1587,7 +1539,7 @@
         <v>12</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>158</v>
@@ -1631,7 +1583,7 @@
         <v>12</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>158</v>
@@ -1675,7 +1627,7 @@
         <v>12</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>158</v>
@@ -1719,7 +1671,7 @@
         <v>12</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>158</v>
@@ -1763,7 +1715,7 @@
         <v>12</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>158</v>
@@ -1807,7 +1759,7 @@
         <v>12</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>158</v>
@@ -1851,7 +1803,7 @@
         <v>12</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H19" s="3" t="s">
         <v>158</v>
@@ -1895,7 +1847,7 @@
         <v>12</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>158</v>
@@ -1939,7 +1891,7 @@
         <v>12</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>158</v>
@@ -1983,7 +1935,7 @@
         <v>12</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>158</v>
@@ -2027,7 +1979,7 @@
         <v>12</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>158</v>
@@ -2071,7 +2023,7 @@
         <v>12</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>158</v>
@@ -2115,7 +2067,7 @@
         <v>12</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H25" s="3" t="s">
         <v>158</v>
@@ -2159,7 +2111,7 @@
         <v>12</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="H26" s="3" t="s">
         <v>158</v>
@@ -2203,7 +2155,7 @@
         <v>12</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H27" s="3" t="s">
         <v>158</v>
@@ -2247,7 +2199,7 @@
         <v>12</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H28" s="3" t="s">
         <v>158</v>
@@ -2291,7 +2243,7 @@
         <v>12</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>158</v>
@@ -2335,7 +2287,7 @@
         <v>12</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H30" s="3" t="s">
         <v>158</v>
@@ -2379,7 +2331,7 @@
         <v>12</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H31" s="3" t="s">
         <v>158</v>
@@ -2423,7 +2375,7 @@
         <v>12</v>
       </c>
       <c r="G32" s="3" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H32" s="3" t="s">
         <v>158</v>
@@ -2449,397 +2401,45 @@
     </row>
     <row r="33" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
-        <v>46208.502451967594</v>
+        <v>46208.498494259256</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D33" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="D33" s="4">
+        <v>82350597713</v>
+      </c>
+      <c r="E33" s="3">
+        <v>31</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="3" t="s">
         <v>161</v>
-      </c>
-      <c r="E33" s="3">
-        <v>35</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>158</v>
       </c>
       <c r="I33" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>14</v>
       </c>
       <c r="K33" s="6" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="L33" s="3" t="s">
-        <v>68</v>
+        <v>150</v>
       </c>
       <c r="M33" s="5" t="s">
         <v>15</v>
       </c>
       <c r="N33" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" ht="22" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
-        <v>46208.686296041662</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="E34" s="3">
-        <v>37</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="I34" s="3">
-        <v>1</v>
-      </c>
-      <c r="J34" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K34" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="L34" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="M34" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N34" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E35" s="3">
-        <v>350</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G35" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I35" s="3">
-        <v>3</v>
-      </c>
-      <c r="J35" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K35" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M35" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N35" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" s="3">
-        <v>3</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G36" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="H36" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I36" s="3">
-        <v>3</v>
-      </c>
-      <c r="J36" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K36" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L36" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M36" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N36" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="E37" s="3">
-        <v>3</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="H37" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I37" s="3">
-        <v>3</v>
-      </c>
-      <c r="J37" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K37" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L37" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M37" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N37" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="8" t="s">
-        <v>178</v>
-      </c>
-      <c r="E38" s="3">
-        <v>3</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="H38" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I38" s="3">
-        <v>3</v>
-      </c>
-      <c r="J38" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K38" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L38" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M38" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N38" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="8" t="s">
-        <v>179</v>
-      </c>
-      <c r="E39" s="3">
-        <v>3</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G39" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="H39" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I39" s="3">
-        <v>3</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K39" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M39" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N39" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
-        <v>46208.502451967594</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="E40" s="3">
-        <v>35</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="I40" s="3">
-        <v>1</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K40" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="M40" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N40" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="41" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
-        <v>46146.267447141203</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="C41" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="8">
-        <v>85253822700</v>
-      </c>
-      <c r="E41" s="3">
-        <v>3</v>
-      </c>
-      <c r="F41" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G41" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="H41" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="I41" s="3">
-        <v>3</v>
-      </c>
-      <c r="J41" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="K41" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L41" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="M41" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="N41" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2876,28 +2476,15 @@
     <hyperlink ref="K30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
     <hyperlink ref="K31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
     <hyperlink ref="K32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="K33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="K34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="M2" r:id="rId34" xr:uid="{0BE99F97-4218-4402-9D78-2E10BC4B924E}"/>
-    <hyperlink ref="M3:M34" r:id="rId35" display="https://drive.google.com/open?id=1ncLerrEwpsR8w5xf8SSXG334E7fOu2R-" xr:uid="{3D388301-D9F2-42DA-A9C0-AABA62A48F07}"/>
-    <hyperlink ref="K35" r:id="rId36" xr:uid="{ACC58351-468A-4939-8ADD-0A99AD034A4C}"/>
-    <hyperlink ref="M35" r:id="rId37" xr:uid="{51268971-6898-4368-8216-B980E5B32BA4}"/>
-    <hyperlink ref="K36" r:id="rId38" xr:uid="{FB207ECB-910A-46DC-B96E-86A5CA0E2842}"/>
-    <hyperlink ref="M36" r:id="rId39" xr:uid="{4F23D56C-A79E-4957-B716-1C96D53704FE}"/>
-    <hyperlink ref="K37" r:id="rId40" xr:uid="{BE5B597F-7643-44C1-909D-533625A1E4AB}"/>
-    <hyperlink ref="M37" r:id="rId41" xr:uid="{9CE496CB-4FB2-49D1-B29F-60A57BF26F9E}"/>
-    <hyperlink ref="K38" r:id="rId42" xr:uid="{B679085D-5408-4DBF-9552-22C63BDCE08C}"/>
-    <hyperlink ref="M38" r:id="rId43" xr:uid="{F5B1B155-0DD2-49EE-BC05-C72A1B03D595}"/>
-    <hyperlink ref="K39" r:id="rId44" xr:uid="{E4C20335-B77C-44A9-AFFF-DBA969766DCF}"/>
-    <hyperlink ref="M39" r:id="rId45" xr:uid="{7F27F93F-40BF-43A3-94C3-0397E3BCBA49}"/>
-    <hyperlink ref="K40" r:id="rId46" xr:uid="{894FE79F-F7F3-401E-97D8-A3F032BD13D1}"/>
-    <hyperlink ref="M40" r:id="rId47" xr:uid="{A8DE7F3A-0698-4A9F-B94C-8857CE31C467}"/>
-    <hyperlink ref="K41" r:id="rId48" xr:uid="{A902B6BA-8088-4ED0-9FA5-B0B94025846C}"/>
-    <hyperlink ref="M41" r:id="rId49" xr:uid="{018ECE75-35A0-4D9B-8718-276209FBE571}"/>
+    <hyperlink ref="M2" r:id="rId32" xr:uid="{0BE99F97-4218-4402-9D78-2E10BC4B924E}"/>
+    <hyperlink ref="M3:M32" r:id="rId33" display="https://drive.google.com/open?id=1ncLerrEwpsR8w5xf8SSXG334E7fOu2R-" xr:uid="{3D388301-D9F2-42DA-A9C0-AABA62A48F07}"/>
+    <hyperlink ref="K33" r:id="rId34" xr:uid="{851E1913-713F-4C17-B7DB-B7941F8C5B36}"/>
+    <hyperlink ref="M33" r:id="rId35" xr:uid="{CB9DF5F6-87C9-414D-AFCE-18762D4E3576}"/>
+    <hyperlink ref="C33" r:id="rId36" xr:uid="{D643F9EB-752C-4B85-A504-CD56BB789434}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId50"/>
+    <tablePart r:id="rId37"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: tambahkan fitur kirim konfirmasi WA ke peserta di dashboard admin
</commit_message>
<xml_diff>
--- a/Informasi Kontak (Jawaban).xlsx
+++ b/Informasi Kontak (Jawaban).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Ruang-Tenang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2FC1366E-38E0-407E-BE5A-BE04AEA3B50F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3F0F0C-8730-470D-B71B-7A8231910E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="171">
   <si>
     <t>Timestamp</t>
   </si>
@@ -523,10 +523,19 @@
     <t>Bukti Follow Akun Instagram "Ruang Tenang Kendari" https://www.instagram.com/ruangtenang.community?igsh=MTNyOW90N2x0bzdjeA==</t>
   </si>
   <si>
-    <t>IkhsandduinRezki</t>
-  </si>
-  <si>
     <t>Ikhsanuddin@gmail.com</t>
+  </si>
+  <si>
+    <t>rezki</t>
+  </si>
+  <si>
+    <t>VVIP</t>
+  </si>
+  <si>
+    <t>rkai</t>
+  </si>
+  <si>
+    <t>vvip</t>
   </si>
 </sst>
 </file>
@@ -977,7 +986,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.90625" customWidth="1"/>
@@ -2404,10 +2413,10 @@
         <v>46208.498494259256</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="C33" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>167</v>
       </c>
       <c r="D33" s="4">
         <v>82350597713</v>
@@ -2419,7 +2428,7 @@
         <v>12</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H33" s="3" t="s">
         <v>158</v>
@@ -2440,6 +2449,50 @@
         <v>15</v>
       </c>
       <c r="N33" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>46208.498494259256</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="D34" s="4">
+        <v>82350597713</v>
+      </c>
+      <c r="E34" s="3">
+        <v>31</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="H34" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="I34" s="3">
+        <v>2</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="K34" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="N34" s="3" t="s">
         <v>17</v>
       </c>
     </row>
@@ -2481,10 +2534,13 @@
     <hyperlink ref="K33" r:id="rId34" xr:uid="{851E1913-713F-4C17-B7DB-B7941F8C5B36}"/>
     <hyperlink ref="M33" r:id="rId35" xr:uid="{CB9DF5F6-87C9-414D-AFCE-18762D4E3576}"/>
     <hyperlink ref="C33" r:id="rId36" xr:uid="{D643F9EB-752C-4B85-A504-CD56BB789434}"/>
+    <hyperlink ref="K34" r:id="rId37" xr:uid="{E64D6B6B-EFC1-4BBD-BF11-7618EE4DD058}"/>
+    <hyperlink ref="M34" r:id="rId38" xr:uid="{78E33065-3D53-4125-AA6C-659132224D82}"/>
+    <hyperlink ref="C34" r:id="rId39" xr:uid="{BCD90EF2-4206-45F0-92FC-D7875B38F498}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId37"/>
+    <tablePart r:id="rId40"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: use absolute URL for Open Graph image to fix WhatsApp preview
</commit_message>
<xml_diff>
--- a/Informasi Kontak (Jawaban).xlsx
+++ b/Informasi Kontak (Jawaban).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\Ruang-Tenang\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF3F0F0C-8730-470D-B71B-7A8231910E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6E5E42-F189-4BB4-B08B-EE2F41BE7854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -535,7 +535,7 @@
     <t>rkai</t>
   </si>
   <si>
-    <t>vvip</t>
+    <t>vip</t>
   </si>
 </sst>
 </file>

</xml_diff>